<commit_message>
Excel data initigration alignment changes
</commit_message>
<xml_diff>
--- a/src/test/resources/data/Datasheet.xlsx
+++ b/src/test/resources/data/Datasheet.xlsx
@@ -4,11 +4,12 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="TESTDATA" sheetId="1" r:id="rId1"/>
-    <sheet name="BOOKAPI" sheetId="2" r:id="rId2"/>
+    <sheet name="Valid_Data" sheetId="1" r:id="rId1"/>
+    <sheet name="InValid_Data" sheetId="3" r:id="rId2"/>
+    <sheet name="TESTDATA" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="7">
   <si>
     <t>userName</t>
   </si>
@@ -34,17 +35,20 @@
     <t>locked_out_user</t>
   </si>
   <si>
-    <t>payload</t>
-  </si>
-  <si>
-    <t>{$$  "userName": "Venki48",$$  "password": "Venki@472"$$}</t>
+    <t>standard_user</t>
+  </si>
+  <si>
+    <t>balasivarathri-wuev@force.com</t>
+  </si>
+  <si>
+    <t>9959@Bala</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -67,6 +71,28 @@
       <name val="JetBrains Mono"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -77,7 +103,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.34998626667073579"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -106,19 +132,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -405,18 +435,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -427,24 +457,65 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="67" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="8.88671875" style="4"/>
+    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="3" t="s">
-        <v>4</v>
+    <row r="1" spans="1:2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" s="4" customFormat="1">
+      <c r="A2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
all working code changes both ui and api
</commit_message>
<xml_diff>
--- a/src/test/resources/data/Datasheet.xlsx
+++ b/src/test/resources/data/Datasheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Valid_Data" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
   <si>
     <t>userName</t>
   </si>
@@ -42,6 +42,15 @@
   </si>
   <si>
     <t>9959@Bala</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>saucelabs</t>
+  </si>
+  <si>
+    <t>salesforce</t>
   </si>
 </sst>
 </file>
@@ -419,7 +428,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -427,26 +436,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -457,26 +472,32 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -487,33 +508,40 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="4" customFormat="1">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:3" s="4" customFormat="1">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="B2" r:id="rId2"/>
+    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="C2" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId3"/>

</xml_diff>